<commit_message>
refactor bad practice code
</commit_message>
<xml_diff>
--- a/src/app/api/[reportId]/Asset_Report.xlsx
+++ b/src/app/api/[reportId]/Asset_Report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29212"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cititex-my.sharepoint.com/personal/chutima_cititex_co_th/Documents/CITITEX Project/Asset Count Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c6058d78e55bea86/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{25C9F719-830E-40C9-88BA-11C8E89A589C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{14DFE9D2-431D-4109-929D-5C6C7AAEF300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{4495CCDA-79BA-4027-8A10-C93A0DF9419C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="24792" windowHeight="14856" xr2:uid="{4495CCDA-79BA-4027-8A10-C93A0DF9419C}"/>
   </bookViews>
   <sheets>
     <sheet name="report" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="21">
   <si>
     <t>CITITEX Group</t>
   </si>
@@ -47,43 +47,28 @@
     <t>Document No.</t>
   </si>
   <si>
-    <t>20250723-01</t>
-  </si>
-  <si>
     <t>Date Count</t>
   </si>
   <si>
     <t>Asset Check Name</t>
   </si>
   <si>
-    <t>Tossawat Umpharote</t>
-  </si>
-  <si>
-    <t>(ชื่อผู้ตรวจ)</t>
-  </si>
-  <si>
     <t>Location</t>
   </si>
   <si>
-    <t>Bangbon / EDP Floor 2</t>
-  </si>
-  <si>
-    <t>(Location ตาม Snipe)</t>
-  </si>
-  <si>
-    <t>Asset Count</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>(จำนวนทรัพย์สินที่มีอยู่ใน location นั้น)</t>
-  </si>
-  <si>
-    <t>(tick manual)</t>
-  </si>
-  <si>
-    <t>ในหน้า Summary Report</t>
+    <t>ทรัพย์สินในระบบทั้งหมด</t>
+  </si>
+  <si>
+    <t>ทรัพย์สินที่ไม่เจอ</t>
+  </si>
+  <si>
+    <t>ทรัพย์สินพบเพิ่มเติม</t>
+  </si>
+  <si>
+    <t>ทรัพย์สินผู้ครอบครองไม่ถูกต้อง</t>
+  </si>
+  <si>
+    <t>ทรัพย์สินเสียหาย</t>
   </si>
   <si>
     <t>No.</t>
@@ -95,31 +80,25 @@
     <t>Asset Name</t>
   </si>
   <si>
-    <t>Assign Name</t>
-  </si>
-  <si>
-    <t>Count Check</t>
-  </si>
-  <si>
-    <t>Assign Not Correct</t>
-  </si>
-  <si>
-    <t>Asset Damaged</t>
-  </si>
-  <si>
-    <t>location</t>
-  </si>
-  <si>
-    <t>CFFL10NB001</t>
-  </si>
-  <si>
-    <t>Notebook Lenovo</t>
-  </si>
-  <si>
-    <t>Tossawat</t>
-  </si>
-  <si>
-    <t>Yes</t>
+    <t>ผู้ครอบครอง</t>
+  </si>
+  <si>
+    <t>ตรวจเจอ</t>
+  </si>
+  <si>
+    <t>ผู้ครองครองไม่ถูกต้อง</t>
+  </si>
+  <si>
+    <t>Location ทรัพย์สิน</t>
+  </si>
+  <si>
+    <t>Location ที่ถูกต้อง</t>
+  </si>
+  <si>
+    <t>ชื่อผู้ครอบครองที่ถูกต้อง</t>
+  </si>
+  <si>
+    <t>Remark</t>
   </si>
 </sst>
 </file>
@@ -185,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -199,6 +178,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -588,169 +568,147 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6458AA90-8DA5-4B1C-AAFD-CB3FE240EC53}">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr defaultRowHeight="16.899999999999999"/>
   <cols>
-    <col min="1" max="1" width="16.875" customWidth="1"/>
+    <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.25" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="35.375" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="20.75" customWidth="1"/>
     <col min="7" max="7" width="17.25" customWidth="1"/>
-    <col min="8" max="8" width="14.875" customWidth="1"/>
+    <col min="8" max="8" width="20.875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.875" customWidth="1"/>
+    <col min="10" max="10" width="15.875" customWidth="1"/>
+    <col min="11" max="11" width="20.875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="39" customHeight="1"/>
-    <row r="2" spans="1:8">
+    <row r="1" spans="1:12" ht="39" customHeight="1"/>
+    <row r="2" spans="1:12">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:12">
       <c r="A3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:12">
       <c r="A5" t="s">
         <v>2</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" t="s">
+      <c r="B6" s="4"/>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="4">
-        <v>45861</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7" t="s">
+      <c r="C7" s="5"/>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" t="s">
         <v>5</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C8" s="5"/>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="B9" s="1"/>
+      <c r="C9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" t="s">
+      <c r="B10" s="7"/>
+      <c r="C10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" t="s">
         <v>8</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B11" s="7"/>
+      <c r="C11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="B12" s="7"/>
+      <c r="C12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9" t="s">
+      <c r="B13" s="7"/>
+      <c r="C13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+    </row>
+    <row r="15" spans="1:12" ht="29.25" customHeight="1">
+      <c r="A15" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B15" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C15" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="D15" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="E15" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" ht="29.25" customHeight="1">
-      <c r="A11" s="3" t="s">
+      <c r="F15" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="G15" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I15" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="J15" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="K15" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="L15" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F11" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="24.95" customHeight="1">
-      <c r="A12" s="2">
+    </row>
+    <row r="16" spans="1:12" ht="24.95" customHeight="1">
+      <c r="A16" s="2">
         <v>1</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="6"/>
-    </row>
-    <row r="13" spans="1:8" ht="24.95" customHeight="1">
-      <c r="A13" s="2">
-        <v>2</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="6"/>
-    </row>
-    <row r="14" spans="1:8" ht="24.95" customHeight="1">
-      <c r="A14" s="2">
-        <v>3</v>
-      </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="6"/>
-    </row>
-    <row r="15" spans="1:8" ht="24.95" customHeight="1">
-      <c r="A15" s="2">
-        <v>4</v>
-      </c>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="6"/>
-    </row>
-    <row r="16" spans="1:8" ht="24.95" customHeight="1">
-      <c r="A16" s="2">
-        <v>5</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -759,10 +717,14 @@
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="6"/>
-    </row>
-    <row r="17" spans="1:8" ht="24.95" customHeight="1">
+      <c r="I16" s="2"/>
+      <c r="J16" s="6"/>
+      <c r="K16" s="6"/>
+      <c r="L16" s="6"/>
+    </row>
+    <row r="17" spans="1:12" ht="24.95" customHeight="1">
       <c r="A17" s="2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -770,11 +732,15 @@
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
-      <c r="H17" s="6"/>
-    </row>
-    <row r="18" spans="1:8" ht="24.95" customHeight="1">
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
+      <c r="L17" s="6"/>
+    </row>
+    <row r="18" spans="1:12" ht="24.95" customHeight="1">
       <c r="A18" s="2">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -783,10 +749,14 @@
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
       <c r="H18" s="6"/>
-    </row>
-    <row r="19" spans="1:8" ht="24.95" customHeight="1">
+      <c r="I18" s="6"/>
+      <c r="J18" s="6"/>
+      <c r="K18" s="6"/>
+      <c r="L18" s="6"/>
+    </row>
+    <row r="19" spans="1:12" ht="24.95" customHeight="1">
       <c r="A19" s="2">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -795,10 +765,14 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="6"/>
-    </row>
-    <row r="20" spans="1:8" ht="24.95" customHeight="1">
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
+      <c r="K19" s="6"/>
+      <c r="L19" s="6"/>
+    </row>
+    <row r="20" spans="1:12" ht="24.95" customHeight="1">
       <c r="A20" s="2">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -807,10 +781,14 @@
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="6"/>
-    </row>
-    <row r="21" spans="1:8" ht="24.95" customHeight="1">
+      <c r="I20" s="6"/>
+      <c r="J20" s="6"/>
+      <c r="K20" s="6"/>
+      <c r="L20" s="6"/>
+    </row>
+    <row r="21" spans="1:12" ht="24.95" customHeight="1">
       <c r="A21" s="2">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -819,6 +797,74 @@
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="6"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="6"/>
+      <c r="K21" s="6"/>
+      <c r="L21" s="6"/>
+    </row>
+    <row r="22" spans="1:12" ht="24.95" customHeight="1">
+      <c r="A22" s="2">
+        <v>7</v>
+      </c>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="6"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="6"/>
+      <c r="K22" s="6"/>
+      <c r="L22" s="6"/>
+    </row>
+    <row r="23" spans="1:12" ht="24.95" customHeight="1">
+      <c r="A23" s="2">
+        <v>8</v>
+      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="6"/>
+      <c r="K23" s="6"/>
+      <c r="L23" s="6"/>
+    </row>
+    <row r="24" spans="1:12" ht="24.95" customHeight="1">
+      <c r="A24" s="2">
+        <v>9</v>
+      </c>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6"/>
+      <c r="J24" s="6"/>
+      <c r="K24" s="6"/>
+      <c r="L24" s="6"/>
+    </row>
+    <row r="25" spans="1:12" ht="24.95" customHeight="1">
+      <c r="A25" s="2">
+        <v>10</v>
+      </c>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="6"/>
+      <c r="J25" s="6"/>
+      <c r="K25" s="6"/>
+      <c r="L25" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>